<commit_message>
feat: atualizar base de dados com oportunidades de 2026
</commit_message>
<xml_diff>
--- a/oportunidades_obras_mt.xlsx
+++ b/oportunidades_obras_mt.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K35"/>
+  <dimension ref="A1:K36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -476,7 +476,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Construção Civil</t>
+          <t>Reforma / Adequação Predial</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -490,7 +490,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>50432.51</v>
+        <v>24373.42</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -499,28 +499,32 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2024-08-20</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr"/>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2026-08-03 08:00</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>MINISTERIO DA JUSTICA E SEGURANCA PUBLICA</t>
+          <t>CONSELHO REGIONAL DE FARMACIA DO ESTADO DE MATO GROSSO</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Construção da fundação para a Guarita Blindada que foi recentemente adquirida pela SR/PF/MT.</t>
+          <t>Contratação de empresa especializada em assessoria técnica nas áreas de Engenharia Civil e/ou Arquitetura para suporte ao Conselho Regional de Farmácia do Estado de Mato Grosso – CRF/MT na revisão, validação e complementação dos documentos técnicos necessários à contratação de empresa para execução da reforma de sua sede, bem como apoio técnico durante o procedimento licitatório</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>08320002906202433</t>
+          <t>024/2026</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>https://pncp.gov.br/app/editais/00394494000136/2024/895</t>
+          <t>https://pncp.gov.br/app/editais/15081680000192/2026/10</t>
         </is>
       </c>
     </row>
@@ -541,7 +545,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>8200</v>
+        <v>17914.5</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -550,44 +554,40 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2024-08-19</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>2024-08-23 08:59</t>
-        </is>
-      </c>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
-          <t>MINISTERIO PUBLICO DA UNIAO</t>
+          <t>CONSELHO REGIONAL DE FARMACIA DO ESTADO DE MATO GROSSO</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Contratação de empresa especializada na prestação de serviço, com o fornecimento de todos os materiais necessários à execução, visando à reforma de mobiliário (mesa de auditório)</t>
+          <t>Contratação de empresa especializada em assessoria técnica nas áreas de Engenharia Civil e/ou Arquitetura para suporte ao Conselho Regional de Farmácia do Estado de Mato Grosso – CRF/MT na revisão, validação e complementação dos documentos técnicos necessários à contratação de empresa para execução da reforma de sua sede, bem como apoio técnico durante o procedimento licitatório</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>564/2024-45</t>
+          <t>029/2026</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>https://pncp.gov.br/app/editais/26989715000102/2024/1581</t>
+          <t>https://pncp.gov.br/app/editais/15081680000192/2026/11</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Manutenção Predial</t>
+          <t>Reforma / Adequação Predial</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>VÁRZEA GRANDE</t>
+          <t>CUIABÁ</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -596,7 +596,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>306297.36</v>
+        <v>812620</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -605,36 +605,35 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2024-08-06</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
-          <t>INSTITUTO FEDERAL DE EDUCACAO, CIENCIA E TECNOLOGIA DE MATO GROSSO</t>
+          <t>FUNDACAO UNIVERSIDADE FEDERAL DE MATO GROSSO</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>ontratação de empresa especializada para prestação dos serviços terceirizados de limpeza, asseio e conservação predial, com dedicação exclusiva de mão de obra, de natureza continuada, para o Campus Várzea Grande do Instituto Federal de Educação, Ciência e Tecnologia de Mato Grosso.
-Carga horária de 44 h semanal.</t>
+          <t>Dispensa de licitação para a contratação da FUNDAÇÃO DE APOIO E DESENVOLVIMENTO DA UFMT - FUNDAÇÃO UNISELVA, para apoio na gestão administrativa e financeira necessária à consecução do projeto intitulado "Curso de Pós-Graduação Lato Sensu Especialização em Direito Tributário e Planejamento Fiscal com Ênfase em Reforma Tributária -EaD", no valor de R$ 812.620,00 (oitocentos e doze mil seiscentos e vinte reais), conforme disposto na Previsão de Receita do Plano de Trabalho aprovado.</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>23749.001007.2024-86</t>
+          <t>23108.004648/2026-08</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>https://pncp.gov.br/app/editais/10784782000150/2024/270</t>
+          <t>https://pncp.gov.br/app/editais/33004540000100/2026/77</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Construção Civil</t>
+          <t>Serviços de Engenharia Geral</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -648,7 +647,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>1156650</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -657,32 +656,28 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2024-07-31</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>2024-08-05 08:59</t>
-        </is>
-      </c>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
-          <t>CONSELHO REGIONAL DE ENGENHARIA E AGRONOMIA DE MATO GROSSO</t>
+          <t>MINISTERIO DA GESTAO E DA INOVACAO EM SERVICOS PUBLICOS</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>O presente instrumento tem por objeto a contratação de empresa para o serviço de aluguel de caçamba bota-fora para descarte de entulhos compreende o fornecimento, entrega, posicionamento, recolhimento e transporte de caçambas metálicas destinadas à coleta e destinação adequada de resíduos da construção civil, bem como resíduos vegetais</t>
+          <t>Contratação direta, por dispensa de licitação, de serviços de engenharia comuns de modernização com substituição integral de 03 (três) elevadores, incluindo manutenção preventiva e corretiva, no Edifício-Sede do MGI/MT.</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>P20240342180</t>
+          <t>10183.000417/2024-19</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>https://pncp.gov.br/app/editais/03471158000138/2024/35</t>
+          <t>https://pncp.gov.br/app/editais/00489828000155/2026/367</t>
         </is>
       </c>
     </row>
@@ -703,7 +698,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>19990</v>
+        <v>428360</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -712,35 +707,35 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2024-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
-          <t>CONSELHO REGIONAL DE MEDICINA DO ESTADO DE MATO GROSSO</t>
+          <t>FUNDACAO UNIVERSIDADE FEDERAL DE MATO GROSSO</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>A contratação de profissional liberal e/ou empresa especializada e habilitada para apresentação técnica e gráfica de projetos de reforma de arquitetura de interiores, seus respectivos projetos complementares e para o acompanhamento/supervisão das obras que serão realizadas na sede do Conselho Regional de Medicina do Estado de Mato Grosso (CRM-MT).</t>
+          <t>Dispensa de licitação para a contratação da FUNDAÇÃO DE APOIO E DESENVOLVIMENTO DA UFMT - FUNDAÇÃO UNISELVA, para apoio na gestão administrativa e financeira necessária à consecução do projeto intitulado "Especialização em Direito Tributário e Planejamento Fiscal com ênfase na Reforma Tributária", no valor de R$ 428.360,00 (quatrocentos e vinte e oito mil, trezentos e sessenta reais)), conforme disposto na Previsão de Receita do Plano de Trabalho aprovado.</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>04/2022</t>
+          <t>23108.004555/2026-75</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>https://pncp.gov.br/app/editais/03008521000183/2022/1</t>
+          <t>https://pncp.gov.br/app/editais/33004540000100/2026/69</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Reforma / Adequação Predial</t>
+          <t>Manutenção Predial</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -754,7 +749,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>2050</v>
+        <v>89999.86</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -763,28 +758,28 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2024-07-01</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
-          <t>MINISTERIO DO TRABALHO E EMPREGO - MTE</t>
+          <t>COMANDO DA MARINHA</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Reforma geral de estante.</t>
+          <t>Contratação de empresa especializada para execução de serviços comuns de engenharia destinados à manutenção predial corretiva e preventiva de Próprios Nacionais Residenciais (PNR) da Agência Fluvial de Cáceres.</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>005/2024</t>
+          <t>63351.000.271/2026-42</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>https://pncp.gov.br/app/editais/37115367000160/2024/85</t>
+          <t>https://pncp.gov.br/app/editais/00394502000144/2026/5960</t>
         </is>
       </c>
     </row>
@@ -805,7 +800,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>4000</v>
+        <v>3978663.88</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -814,35 +809,35 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2024-06-28</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
-          <t>COMANDO DO EXERCITO</t>
+          <t>PROCURADORIA GERAL DE JUSTICA DO ESTADO DE MATO GROSSO</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Contratação do serviço de manutenção de prensa hidráulica do 44°BIMtz.</t>
+          <t>Fornecer sistemas de climatização do tipo VRF, compreendendo unidades condensadoras, unidades evaporadoras e acessórios necessários para atender à Sede das Promotorias de Justiça da Capital, conforme condições e exigências estabelecidas no Termo de Referência.</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>64104003872202349</t>
+          <t>20.14.0001.0002470/2026-66</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>https://pncp.gov.br/app/editais/00394452000103/2024/11723</t>
+          <t>https://pncp.gov.br/app/editais/14921092000157/2026/81</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Instalações / Climatização</t>
+          <t>Reforma / Adequação Predial</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -856,7 +851,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>4318</v>
+        <v>0</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -865,32 +860,32 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2024-06-20</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2024-06-27 07:59</t>
+          <t>2026-06-03 08:00</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>COMANDO DO EXERCITO</t>
+          <t>PROCURADORIA GERAL DE JUSTICA DO ESTADO DE MATO GROSSO</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Manutenção de prensa hidráulica (SFPC - 44°BITMZ):  1. Montagem e desmontagem (mão de obra)  2. Reparo/troca do pistão de descida (cilindro hidráulico)  3. Limpeza e higienização do reservatório de óleo  4. Troca de óleo  5. Reparo ou troca de porcas das mangueiras de óleo</t>
+          <t>Execução  de reforma  e  modernização  da cobertura  da  Sede  das  Promotorias  da  Capital,  incluindo  instalação  de  estrutura  metálica, plataformas  metálicas, forro do  3º andar,  vedação  da pele  de  vidro  horizontal e  adequação das  instalações  elétricas  dos  circuitos  de  climatização,conforme  condições  e  exigências estabelecidas neste instrumento.</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>64104003996202413</t>
+          <t>20.14.0001.0002463/2026-61</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>https://pncp.gov.br/app/editais/00394452000103/2024/10986</t>
+          <t>https://pncp.gov.br/app/editais/14921092000157/2026/77</t>
         </is>
       </c>
     </row>
@@ -911,7 +906,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>17430</v>
+        <v>2367</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -920,28 +915,28 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2024-06-12</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
-          <t>MINISTERIO DO TRABALHO E EMPREGO - MTE</t>
+          <t>JUSTICA FEDERAL DE PRIMEIRA INSTANCIA</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Contratação de Prestador de Serviço em Reforma e Manutenção de Cadeiras e Longarinas.</t>
+          <t>Contratação de empresa especializada com fornecimento de mão de obra para serviços de  Reinstalação de porta giratória com detector de metais em caráter de urgência, visando garantir a continuidade dos serviços judiciários e a segurança das instalações  após a reforma de pisos da Subseção Judiciária de Cáceres</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>002/2024</t>
+          <t>21881920264018009</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>https://pncp.gov.br/app/editais/37115367000160/2024/70</t>
+          <t>https://pncp.gov.br/app/editais/00508903000188/2026/1014</t>
         </is>
       </c>
     </row>
@@ -962,7 +957,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>349898.88</v>
+        <v>89999.86</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -971,35 +966,39 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2024-05-13</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr"/>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>2026-06-02 09:00</t>
+        </is>
+      </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>FUNDACAO UNIVERSIDADE FEDERAL DE MATO GROSSO</t>
+          <t>COMANDO DA MARINHA</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Contratação EMERGENCIAL de empresa especializada na prestação de serviços continuados de limpeza, asseio e conservação, com fornecimento de mão de obra, saneantes, equipamentos/utensílios e materiais de consumo, serviço de manutenção predial e conservação conforme TR 30/2024 . Processo 23108.026580/2024-48.</t>
+          <t>Contratação de empresa especializada para execução de serviços comuns de engenharia destinados à manutenção predial corretiva e preventiva de Próprios Nacionais Residenciais (PNR) da Agência Fluvial de Cáceres.</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>23108.026580/2024-48</t>
+          <t>63351.000.271/2026-42</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>https://pncp.gov.br/app/editais/33004540000100/2024/18</t>
+          <t>https://pncp.gov.br/app/editais/00394502000144/2026/5283</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Instalações / Climatização</t>
+          <t>Pavimentação / Infraestrutura</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1013,7 +1012,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>1670</v>
+        <v>29362.8</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -1022,39 +1021,39 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2024-05-08</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2024-05-15 07:59</t>
+          <t>2026-05-25 09:00</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>MINISTERIO PUBLICO DA UNIAO</t>
+          <t>CONSELHO REGIONAL DE ENGENHARIA E AGRONOMIA DE MATO GROSSO</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>CAFETEIRA ELÉTRICA, automática, prepara e mantém o café aquecido, capacidade mínima 6 litros, em aço inoxidável 430, termostato, bivolt 110/220v, ou 110v, aro coador em aço 304, dispensa o uso de coador em pano ou papel, corpo em aço escovado, pingadeira removível para facilitar a limpeza, lâmpada indicadora de aquecimento, potência mínima de 1000W. Certificação do INMETRO. Garantia de 12 meses. Marca de referência: MARCHESONI, equivalente ou de melhor qualidade.</t>
+          <t>Contratação de empresa especializada em engenharia para elaboração dos projetos básico e executivo da futura Inspetoria do CREA-MT em Alta Floresta/MT, incluindo levantamento planialtimétrico, planilha orçamentária, memoriais descritivos, compatibilização de projetos e aprovação junto aos órgãos competentes, contemplando as disciplinas de arquitetura, estrutural, instalações elétricas, hidrossanitárias, drenagem, lógica e telecomunicações, climatização entre outros.</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>320/2024-37</t>
+          <t>P2026/023895-8</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>https://pncp.gov.br/app/editais/26989715000102/2024/613</t>
+          <t>https://pncp.gov.br/app/editais/03471158000138/2026/22</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Instalações / Climatização</t>
+          <t>Serviços de Engenharia Geral</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1068,7 +1067,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>49355</v>
+        <v>80422.27</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -1077,35 +1076,39 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2024-04-24</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr"/>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>2026-05-22 09:00</t>
+        </is>
+      </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>INSTITUTO FEDERAL DE EDUCACAO, CIENCIA E TECNOLOGIA DE MATO GROSSO</t>
+          <t>DNIT-DEPARTAMENTO NACIONAL DE INFRAEST DE TRANSPORTES</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Contratação de prestação de serviço de manutenção preventiva e corretiva em aparelhos de climatização</t>
+          <t>Contratação de serviço de engenharia para a implantação completa do Sistema de Segurança Contra Incêndio e Pânico na sede da Superintendência Regional do DNIT/MT, incluindo fornecimento integral de materiais, mão de obra e a obtenção do Alvará de Segurança Contra Incêndio e Pânico (ASCIP) junto ao Corpo de Bombeiros Militar de Mato Grosso.</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>23750.000115.2024-01</t>
+          <t>50611.002326/2025-18</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>https://pncp.gov.br/app/editais/10784782000150/2024/117</t>
+          <t>https://pncp.gov.br/app/editais/04892707002235/2026/24</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Instalações / Climatização</t>
+          <t>Construção Civil</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1119,7 +1122,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>4898</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -1128,39 +1131,40 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2024-04-23</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2024-04-26 07:59</t>
+          <t>2026-05-11 08:00</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>PROCURADORIA GERAL DE JUSTICA DO ESTADO DE MATO GROSSO</t>
+          <t>COMANDO DO EXERCITO</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Contratação de empresa especializada para prestação de serviço de manutenção corretiva, com fornecimento de peças, para o sistema de geração de energia elétrica fotovoltaica presente na Sede das Promotorias da Infância e Juventude de Cuiabá, conforme condições e exigências estabelecidas neste instrumento.</t>
+          <t>Cortador manual de bloco de concreto tipo paver intertravado, para utilização em obras de pavimentação, com sistema de corte por alavanca e lâminas/elementos de corte apropriados ao material (concreto). Capacidade de corte compatível com pavers com altura/espessura mínima de 5 cm e máxima de 12 cm, ou superior Largura útil/capacidade 
+dimensional: capacidade de corte para blocos com largura de até 33 cm, ou superior. Construção: estrutura robusta em material metálico.</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>000303-001/2024</t>
+          <t>64047.000140/2026-71</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>https://pncp.gov.br/app/editais/14921092000157/2024/74</t>
+          <t>https://pncp.gov.br/app/editais/00394452000103/2026/8886</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Instalações / Climatização</t>
+          <t>Manutenção Predial</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1174,7 +1178,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>23110.8</v>
+        <v>14400</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -1183,32 +1187,28 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2024-04-18</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>2024-04-23 08:59</t>
-        </is>
-      </c>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
-          <t>CONSELHO REGIONAL DE ENGENHARIA E AGRONOMIA DE MATO GROSSO</t>
+          <t>CONSELHO REGIONAL DE FISIOTERAPIA E TERAPIA OCUPACIONAL</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Contratação de cafeteira elétrica e garrafa de café para atender as necessidades do CREA-MT.</t>
+          <t>Serviço de limpeza, asseio, conservação predial e copeiragem, com sede em Cuiabá, e desempenhar serviços na sede do CREFITO-9 em Cuiabá-MT, com fornecimento de mão de obra em regime de dedicação exclusiva de 01 (um) funcionário. Escala de trabalho: 30h (trinta) horas semanais, sendo: de segunda-feira à sexta-feira das 07:30 - 13:45 (com 15 minutos de intervalo) .Rua H, Quadra 04, Setor A, Lote 02, Centro Político Administrativo, Cuiabá - MT, CEP 78049-911</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>20240163987</t>
+          <t>09.0913.000008/2026-13</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>https://pncp.gov.br/app/editais/03471158000138/2024/14</t>
+          <t>https://pncp.gov.br/app/editais/00577473000156/2026/4</t>
         </is>
       </c>
     </row>
@@ -1229,7 +1229,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>27280</v>
+        <v>8040</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -1238,32 +1238,28 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2024-04-11</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>2024-04-17 07:59</t>
-        </is>
-      </c>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
-          <t>MINISTERIO DA JUSTICA E SEGURANCA PUBLICA</t>
+          <t>JUSTICA FEDERAL DE PRIMEIRA INSTANCIA</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Serviços de desinfestação, desinsetização, desratização, descupinização e combate a escorpiões nas instalações dos edifícios em uso pela Polícia Federal em Mato Grosso (áreas internas e externas), com fornecimento de material, ferramentas, utensílios e equipamentos, e deverão ser realizados em todos os ambientes dos respectivos prédios, tais como: edificações principais e secundárias, subestação de energia elétrica, caixas de gordura e caixas de esgoto, lixeiras, e outros</t>
+          <t>Fornecimento de mola piso hidráulica em aço inox, capacidade para 180 kg, com tampa, eixo e dobradiça para a Subseção Judiciária de Cáceres - Mato Grosso</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>08320000534202419</t>
+          <t>13654520264018009</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>https://pncp.gov.br/app/editais/00394494000136/2024/268</t>
+          <t>https://pncp.gov.br/app/editais/00508903000188/2026/563</t>
         </is>
       </c>
     </row>
@@ -1284,7 +1280,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>123900</v>
+        <v>34169.86</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -1293,35 +1289,35 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2024-04-09</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
-          <t>PROCURADORIA GERAL DE JUSTICA DO ESTADO DE MATO GROSSO</t>
+          <t>CONSELHO REGIONAL DE ADMINISTRACAO MATO GROSSO</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Contratação, por DISPENSA DE LICITAÇÃO, da empresa J. L. M. CONSTRUTORA E PROJETOS LTDA, CNPJ nº 17.107.098/0001-83, no valor total de R$ 123.900,00 (cento e vinte e três mil e novecentos  reais), para prestação de serviços de reforma predial emergencial, especificamente reforma completa da cobertura da Sede das Promotorias de Justiça de Tangará da Serra-MT, sem alteração da área construída, com fornecimento de materiais e mão de obra.</t>
+          <t>Contratação de empresa especializada para elaboração de projetos de arquitetura, arquitetura de interiores e projetos complementares, incluindo levantamento técnico, identificação de patologias existentes na edificação, consolidação de projetos já executados, elaboração de memoriais descritivos, orçamento e demais documentos técnicos necessários para subsidiar a futura licitação das obras de manutenção, adequação e reforma da sede do CRA-MT.</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>20.14.0001.0001212/2024-88</t>
+          <t>476909.000142/2026-31</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>https://pncp.gov.br/app/editais/14921092000157/2024/60</t>
+          <t>https://pncp.gov.br/app/editais/26562892000108/2026/6</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Instalações / Climatização</t>
+          <t>Reforma / Adequação Predial</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1335,7 +1331,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0</v>
+        <v>26836.47</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -1344,39 +1340,39 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2024-03-13</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2024-03-20 07:59</t>
+          <t>2026-03-17 08:00</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>CONSELHO REGIONAL DE FARMACIA DO ESTADO DE MATO GROSSO</t>
+          <t>CONSELHO REGIONAL DE EDUCACAO FISICA DA 17A REGIAO - ESTADO DE MATO GROSSO</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>O objeto da presente dispensa é aquisição, instalação e remanejamento de equipamentos de ar condicionado destinados à climatização dos ambientes internos do Conselho Regional de Farmácia do Estado de Mato Grosso (CRF/MT), nos termos da tabela a seguir, conforme condições, quantidades e exigências estabelecidas neste Aviso de Contratação Direta e seus anexos</t>
+          <t>Contratação de serviços de engenharia para Elaboração/Análise de Projeto de reforma e adequação sede e , nos termos da tabela abaixo, conforme condições estudo de viabilidade junto a Prefeitura de Cuiabá/MT e exigências estabelecidas neste instrumento.</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>011/2024</t>
+          <t>005/2026</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>https://pncp.gov.br/app/editais/15081680000192/2024/3</t>
+          <t>https://pncp.gov.br/app/editais/23411944000157/2026/8</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Pavimentação / Infraestrutura</t>
+          <t>Instalações / Climatização</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1390,7 +1386,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>61703291.52</v>
+        <v>1733122.72</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -1399,35 +1395,35 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2024-03-05</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
-          <t>DNIT-DEPARTAMENTO NACIONAL DE INFRAEST DE TRANSPORTES</t>
+          <t>EMPRESA BRASILEIRA DE SERVICOS HOSPITALARES - EBSERH</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Execução dos serviços emergenciais de recuperação na Rodovia Federal BR-158/MT; Trecho: Divisa PA/MT (Início das Obras de Pavimentação) - Divisa MT/GO (Fim Ponte s/Rio Araguaia); Subtrecho: Fim das Obras de Pavimentação - Entr. MT-322(B)/433 (Alô Brasil), Segmento: km 201,20 ao km 330,60; Pontos Críticos: km 202,800 ao km 322,900 e local no km 278,500 (Bueiro); Código SNV: 158BMT0205 - 158BMT0215.</t>
+          <t>Consumo estimado do serviço de energia elétrica para programação orçamentária e publicação da despesa em 2026.</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>50611000198/2024-97</t>
+          <t>23532.000958/2026-35</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>https://pncp.gov.br/app/editais/04892707000100/2025/2</t>
+          <t>https://pncp.gov.br/app/editais/15126437000305/2026/422</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Pavimentação / Infraestrutura</t>
+          <t>Instalações / Climatização</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1441,7 +1437,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>61703291.52</v>
+        <v>5000</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -1450,49 +1446,49 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2024-03-05</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
-          <t>DNIT-DEPARTAMENTO NACIONAL DE INFRAEST DE TRANSPORTES</t>
+          <t>INSTITUTO DO PATRIMONIO HISTORICO E ARTISTICO NACIONAL</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Execução dos serviços emergenciais de recuperação na Rodovia Federal BR-158/MT; Trecho: Divisa PA/MT (Início das Obras de Pavimentação) - Divisa MT/GO (Fim Ponte s/Rio Araguaia); Subtrecho: Fim das Obras de Pavimentação - Entr. MT-322(B)/433 (Alô Brasil), Segmento: km 201,20 ao km 330,60; Pontos Críticos: km 202,800 ao km 322,900 e local no km 278,500 (Bueiro); Código SNV: 158BMT0205 - 158BMT0215</t>
+          <t>Substituição de dois disjuntores no prédio que abriga o IPHAN-MT para reestabelecimento da energia elétrica.</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>50611000198202497</t>
+          <t>01425.000004/2026-15</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>https://pncp.gov.br/app/editais/04892707000100/2024/106</t>
+          <t>https://pncp.gov.br/app/editais/26474056000171/2026/33</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Construção Civil</t>
+          <t>Instalações / Climatização</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>CUIABÁ</t>
+          <t>BARRA DO GARÇAS</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>0</v>
+        <v>63500</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -1501,32 +1497,32 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2024-02-29</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2024-03-07 08:59</t>
+          <t>2026-07-24 08:30</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>CONSELHO REGIONAL DE ENGENHARIA E AGRONOMIA DE MATO GROSSO</t>
+          <t>INSTITUTO FEDERAL DE EDUCACAO, CIENCIA E TECNOLOGIA DE MATO GROSSO</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Levantamento planialtimétrico do terreno, elaboração de projeto executivo de arquitetura com base em anteprojeto elaborado pelo setor de projetos do crea-mt, elaboração de projetos complementares, orçamento completo com planilha geral de quantitativos e respectivos memoriais descritivos, para futura construção da inspetoria do crea-mt no município de alta floresta.</t>
+          <t>Contratação de serviços de remoção e instalação de equipamentos de climatização, com fornecimento de peças.</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>P20240019690</t>
+          <t>23189.000612.2026-94</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>https://pncp.gov.br/app/editais/03471158000138/2024/8</t>
+          <t>https://pncp.gov.br/app/editais/10784782000150/2026/258</t>
         </is>
       </c>
     </row>
@@ -1538,16 +1534,16 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>CUIABÁ</t>
+          <t>RONDONÓPOLIS</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>50789.12</v>
+        <v>3432.6</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -1556,32 +1552,34 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2024-02-09</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2024-02-27 08:59</t>
+          <t>2026-07-03 08:00</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>CONSELHO REGIONAL DE ENGENHARIA E AGRONOMIA DE MATO GROSSO</t>
+          <t>COMANDO DO EXERCITO</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Levantamento Planialtimétrico do terreno, Elaboração de projeto executivo de arquitetura com base em anteprojeto elaborado pelo setor de projetos do CREA-MT, Elaboração de projetos complementares, orçamento completo com planilha geral de quantitativos e respectivos memoriais descritivos, para construção da Inspetoria do CREA-MT no município de Alta Floresta. O projeto deverá atender todas as legislações municipais e estaduais para a aprovação junto aos  órgãos competentes.</t>
+          <t>1. Tijolo, Material: Barro Cozido,Tipo: Maciço, Comprimento: 21, Largura: 10, Espessura: 5,50,  Cor:  Vermelha, Aplicação: Construção Civil.
+2. Argamassa Refrataria - Componentes: Argila Refratária,  Sílica, Cimento Refratário E, Uso: Altas Temperaturas, Aplicação: Churrasqueiras, Lareiras, Fornos E Fogões A Lenha.
+3. Tipo Madeira: Perobinha, Formato: Viga, Comprimento: 6, Largura: 16, Espessura: 6</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>P20240019690</t>
+          <t>64553.002892/2026-57</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>https://pncp.gov.br/app/editais/03471158000138/2024/5</t>
+          <t>https://pncp.gov.br/app/editais/00394452000103/2026/12334</t>
         </is>
       </c>
     </row>
@@ -1593,16 +1591,16 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>CUIABÁ</t>
+          <t>SINOP</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>775000</v>
+        <v>0.0001</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -1611,49 +1609,53 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2024-02-09</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr"/>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>2026-06-30 08:00</t>
+        </is>
+      </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>PROCURADORIA GERAL DE JUSTICA DO ESTADO DE MATO GROSSO</t>
+          <t>EMPRESA BRASILEIRA DE PESQUISA AGROPECUARIA</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Contratação emergencial de empresa especializada para a prestação de serviços de manutenção preventiva, corretiva, instalação, desinstalação e/ou remanejamento de aparelhos/equipamentos, com fornecimento de insumos (peças, materiais e outros mais), serviços e mão de obra, sob demanda, nos sistemas de climatização e refrigeração das unidades do Ministério Público do Estado de Mato Grosso do Polo institucional 1 - Cuiabá, com valor total de R$ 775.000,00 (setecentos e setenta e cinco mil reais)</t>
+          <t>Contratação de empresa especializada para prestação de serviços de desinstalação de sistema antigo e instalação de novo Sistema de Climatização de Teto para veículo tipo Micro-ônibus, com fornecimento integral do equipamento e insumos.</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>20.14.0001.0008355/2023-66</t>
+          <t>21155.000792/2026-76</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>https://pncp.gov.br/app/editais/14921092000157/2024/22</t>
+          <t>https://pncp.gov.br/app/editais/00348003000110/2026/429</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Manutenção Predial</t>
+          <t>Serviços de Engenharia Geral</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>CUIABÁ</t>
+          <t>JUÍNA</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>14849.25</v>
+        <v>42032.64</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1662,10 +1664,14 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2024-02-02</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr"/>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>2026-06-11 08:00</t>
+        </is>
+      </c>
       <c r="H24" t="inlineStr">
         <is>
           <t>INSTITUTO FEDERAL DE EDUCACAO, CIENCIA E TECNOLOGIA DE MATO GROSSO</t>
@@ -1673,24 +1679,24 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Contratação emergencial de empresa para prestação de serviços contínuos, com dedicação exclusiva de mão de obra, de limpeza, asseio e conservação predial, com fornecimento de uniformes e EPIs - IFMT TGA</t>
+          <t>Contratação de empresa para prestação de serviço técnico especializado de apoio à fiscalização de obras e serviços de engenharia para atender as demandas do IFMT - Campus Juína</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>23753.000033.2024-28</t>
+          <t>23195.000871.2025-55</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>https://pncp.gov.br/app/editais/10784782000150/2024/23</t>
+          <t>https://pncp.gov.br/app/editais/10784782000150/2026/180</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Manutenção Predial</t>
+          <t>Construção Civil</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1704,7 +1710,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>12455.7</v>
+        <v>7800</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -1713,40 +1719,44 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2024-08-22</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr"/>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>2026-06-08 12:00</t>
+        </is>
+      </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>INSTITUTO FEDERAL DE EDUCACAO, CIENCIA E TECNOLOGIA DE MATO GROSSO</t>
+          <t>COMANDO DO EXERCITO</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Aquisição EMERGENCIAL de materiais de manutenção predial para reparos URGENTES nas estruturas do IFMT Campus Cáceres - Prof. Olegário Baldo.</t>
+          <t>Materiais de construção destinados à execução de reparos, recomposição e conservação de estruturas prediais.</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>23191.000775.2024-66</t>
+          <t xml:space="preserve"> 64054.006070/2026-76</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>https://pncp.gov.br/app/editais/10784782000150/2024/299</t>
+          <t>https://pncp.gov.br/app/editais/00394452000103/2026/10772</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Manutenção Predial</t>
+          <t>Reforma / Adequação Predial</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>JUÍNA</t>
+          <t>SINOP</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1755,7 +1765,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>1557.4</v>
+        <v>15530</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -1764,40 +1774,40 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2024-06-25</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr">
         <is>
-          <t>INSTITUTO FEDERAL DE EDUCACAO, CIENCIA E TECNOLOGIA DE MATO GROSSO</t>
+          <t>EMPRESA BRASILEIRA DE PESQUISA AGROPECUARIA</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Aquisição materiais e ferramentas para manutenção predial.</t>
+          <t>Serviços de tapeçaria e reforma de mobiliário para a restauração completa dos estofados da sede da Embrapa Agrossilvipastoril. O serviço compreende a substituição de revestimentos e preenchimento com espuma.</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>23195.000438.2024-39</t>
+          <t>21155.000535/2026-34</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>https://pncp.gov.br/app/editais/10784782000150/2024/197</t>
+          <t>https://pncp.gov.br/app/editais/00348003000110/2026/229</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Manutenção Predial</t>
+          <t>Instalações / Climatização</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>RIBEIRÃO CASCALHEIRA</t>
+          <t>RONDONÓPOLIS</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1806,7 +1816,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>19999</v>
+        <v>2066.66</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1815,40 +1825,46 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2024-06-11</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr"/>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>2026-05-14 08:00</t>
+        </is>
+      </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>FUNDACAO NACIONAL DO INDIO</t>
+          <t>COMANDO DO EXERCITO</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Contratação de empresa especializada na prestação dos serviços de manutenção predial, com fornecimento dos materiais e dos insumos necessários, além dos equipamentos e mão-de-obra, referente à pintura e revitalização de alvenaria.</t>
+          <t>1. Manutenção bebedouro da guarda; troca de motor; higienização; troca do dreno; reparo fiação elétrica; troca flange ½ do bebedouro; rebites na tampa.
+2. Manutenção bebedouro da 1ª Bateria de Obuses; troca do ventilador; higienização; rebites na tampa.
+3. Manutenção bebedouro do PRM; troca do ventilador; higienização; rebites na tampa.</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>08100.000242/2024-62</t>
+          <t>64553.001878/2026-36</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>https://pncp.gov.br/app/editais/00059311000126/2024/247</t>
+          <t>https://pncp.gov.br/app/editais/00394452000103/2026/9149</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Reforma / Adequação Predial</t>
+          <t>Instalações / Climatização</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>DIAMANTINO</t>
+          <t>RONDONÓPOLIS</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1857,7 +1873,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>111793.08</v>
+        <v>2165.63</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1866,32 +1882,32 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2024-05-24</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>2024-06-03 07:59</t>
+          <t>2026-05-08 08:00</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>ESTADO DE MATO GROSSO</t>
+          <t>COMANDO DO EXERCITO</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Contratação de empresa especializada para contratação de empresa especializada em elaboração de anteprojeto, projeto básico e projeto executivo, incluindo memorial descritivo/caderno de especificações e encargos, planilha de quantitativos e preços, projetos complementares de engenharia e cronograma Físico-financeiro para a reforma/ampliação da Câmara Municipal de Diamantino-MT.</t>
+          <t>1. Cafeteira Elétrica Capacidade: 1,50L, Voltagem: 220 V, Normas Técnicas: Aisi 304, Características Adicionais: Compacta/ Café Expresso E Capuccino/ Moedor/ Reserva</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>184/2024</t>
+          <t>64553.001811/2026-00</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>https://pncp.gov.br/app/editais/03507415000144/2024/119</t>
+          <t>https://pncp.gov.br/app/editais/00394452000103/2026/8783</t>
         </is>
       </c>
     </row>
@@ -1903,7 +1919,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>JUÍNA</t>
+          <t>SINOP</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1912,7 +1928,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>158833.2</v>
+        <v>241782.12</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1921,7 +1937,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2024-05-10</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="G29" t="inlineStr"/>
@@ -1932,33 +1948,29 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>O contrato com a empresa atual prestadora de serviços de oficial de
-serviços gerais (pedreiros) tem seu vencimento em 15 de março de 2024tem seu vencimento em 15 de março . O contrato não pode ser
-renovado porque a empresa não tem interesse na renovação, e não possuímos ata vigente para contratação. O
-Campus Juína depende dessa mão de obra terceirizada para a manutenção predial preventiva e corretiva.
-Considerando a importância do serviço, bem como a impossibilidade do campus fica sem a prestaçã</t>
+          <t>Contratação de pessoa Jurídica para prestação de serviços terceirizados de natureza continuada de limpeza, conservação predial, asseio, com fornecimento de mão de obra em dedicação exclusiva, uniformes, materiais, utensílios e equipamentos para atendimento ao IFMT- Instituto Federal de Educação, Ciência e Tecnologia de Mato Grosso - Campus Sinop.</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>23195.000074.2024-97</t>
+          <t>23752.000517.2025-68</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>https://pncp.gov.br/app/editais/10784782000150/2024/134</t>
+          <t>https://pncp.gov.br/app/editais/10784782000150/2026/120</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Reforma / Adequação Predial</t>
+          <t>Instalações / Climatização</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>SÃO FÉLIX DO ARAGUAIA</t>
+          <t>SORRISO</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1967,7 +1979,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>73997.34</v>
+        <v>130880</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1976,44 +1988,44 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>2024-03-26</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>2024-04-11 09:59</t>
+          <t>2026-03-30 09:00</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>MINISTERIO DA SAUDE</t>
+          <t>INSTITUTO FEDERAL DE EDUCACAO, CIENCIA E TECNOLOGIA DE MATO GROSSO</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Contratação de empresa especializada em reforma e manutenção predial, com a inclusão de material,  para execução de obra de reforma do antigo polo base de saúde indígena localizado no município de Confresa - MT, jurisdicionado ao DSEI Araguaia/SESAI/MS,  conforme condições, quantidades e exigências estabelecidas neste instrumento e seus anexos.</t>
+          <t>Serviço de Engenharia para Apoio/consultoria na Execução de Obras e Projetos de Correção e Melhorias na Rede Elétrica para o IFMT Campus Sorriso Sede e Fazenda Experimental.</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>25045001048202344</t>
+          <t>23444.000863.2025-20</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>https://pncp.gov.br/app/editais/00394544000185/2024/318</t>
+          <t>https://pncp.gov.br/app/editais/10784782000150/2026/93</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Instalações / Climatização</t>
+          <t>Construção Civil</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>CÁCERES</t>
+          <t>JUÍNA</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -2022,7 +2034,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>7970</v>
+        <v>34611</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -2031,12 +2043,12 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>2024-03-21</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>2024-03-26 07:59</t>
+          <t>2026-03-20 08:00</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -2046,24 +2058,24 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Contratação de serviços de manutenção em aparelhos de climatização do refeitório do IFMT Campus Cáceres.</t>
+          <t>Aquisição materiais de construção e materiais elétricos para atender as demandas do IFMT - Campus Juína</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>23191000941202343</t>
+          <t>23195.000096.2026-19</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>https://pncp.gov.br/app/editais/10784782000150/2024/92</t>
+          <t>https://pncp.gov.br/app/editais/10784782000150/2026/83</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Construção Civil</t>
+          <t>Instalações / Climatização</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2077,7 +2089,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>19947.24</v>
+        <v>2421.88</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -2086,10 +2098,14 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>2024-03-13</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr"/>
+          <t>2026-03-10</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>2026-03-16 08:00</t>
+        </is>
+      </c>
       <c r="H32" t="inlineStr">
         <is>
           <t>COMANDO DO EXERCITO</t>
@@ -2097,17 +2113,17 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Dispensa de Licitação Eletrônica para compra de materiais de construção e elétrica do 18ºGAC</t>
+          <t>Cafeteira Elétrica Material: Aço Inox Aisi 304, Aplicação: Industrial, Capacidade: 8 L, Voltagem: 220 V, Características Adicionais: Caldeira 14l Água, Termostato, Nível E Torneira, Potência: 1.300</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>64553.000621/2024-03</t>
+          <t>64553.000994/2026-38</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>https://pncp.gov.br/app/editais/00394452000103/2024/2186</t>
+          <t>https://pncp.gov.br/app/editais/00394452000103/2026/5508</t>
         </is>
       </c>
     </row>
@@ -2128,7 +2144,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>2335.34</v>
+        <v>10078.17</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -2137,7 +2153,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2024-02-20</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="G33" t="inlineStr"/>
@@ -2148,29 +2164,29 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Aquisição emergencial de materiais elétricos para troca do cabeamento e outros componentes para recuperação da rede elétrica das salas de engenharia florestal, afetadas pela tempestade ocorrida no IFMT Campus Cáceres - Prof. Olegário Baldo.</t>
+          <t>Aquisição emergencial de cabos elétricos e conectores para restabelecimento da energia elétrica no IFMT – Campus Cáceres Professor Olegário Baldo.</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>23191.000148.2024-25</t>
+          <t>23191.000235.2026-44</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>https://pncp.gov.br/app/editais/10784782000150/2024/43</t>
+          <t>https://pncp.gov.br/app/editais/10784782000150/2026/73</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Serviços de Engenharia Geral</t>
+          <t>Pavimentação / Infraestrutura</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>JUARA</t>
+          <t>RONDONÓPOLIS</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -2179,7 +2195,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>14267.12</v>
+        <v>31325.28</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -2188,83 +2204,138 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>2024-01-31</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr"/>
+          <t>2026-02-27</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>2026-03-04 08:00</t>
+        </is>
+      </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>ESTADO DE MATO GROSSO</t>
+          <t>INSTITUTO FEDERAL DE EDUCACAO, CIENCIA E TECNOLOGIA DE MATO GROSSO</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>Contratação de empresa especializada para prestação de serviços de engenharia para assessoramento, acompanhamento e fiscalização dos serviços de execução do projeto estrutural metálico de cobertura com telha isotérmica, projeto de águas pluviais e contrapiso no prédio da Câmara de Juara, conforme Contrato nº 014/2023.</t>
+          <t>Contratação de empresa especializada para execução de serviços comuns de engenharia, de natureza não contínua, destinados à Manutenção corretiva da cobertura, adequação do sistema de drenagem pluvial, bem como à impermeabilização de cisterna de água IFMT Campus Rondonópolis.</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>001/2024</t>
+          <t>23196.001773.2025-25</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>https://pncp.gov.br/app/editais/03507415000144/2024/19</t>
+          <t>https://pncp.gov.br/app/editais/10784782000150/2026/59</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
+          <t>Reforma / Adequação Predial</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>CÁCERES</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>121487.33</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Dispensa</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>2026-02-24</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>2026-03-10 08:00</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>INSTITUTO FEDERAL DE EDUCACAO, CIENCIA E TECNOLOGIA DE MATO GROSSO</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Contratação de empresa especializada para prestação de serviços de engenharia visando a inspeção técnica, emissão de laudo e elaboração de projetos de reforma elétrica (Baixa Tensão, Média Tensão) para o IFMT Campus Cáceres.</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>23191.001278.2025-66</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>https://pncp.gov.br/app/editais/10784782000150/2026/55</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
           <t>Instalações / Climatização</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>PRIMAVERA DO LESTE</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>CONFRESA</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
-      <c r="D35" t="n">
-        <v>53286.2</v>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>Dispensa</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>2024-01-24</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>2024-01-29 07:59</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
+      <c r="D36" t="n">
+        <v>34814.91</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Dispensa</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr">
         <is>
           <t>INSTITUTO FEDERAL DE EDUCACAO, CIENCIA E TECNOLOGIA DE MATO GROSSO</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>Contratação de serviços de manutenção preventiva e corretiva em aparelhos de climatização, com fornecimento de peças para atender as necessidades do IFMT campus Primavera do Leste.</t>
-        </is>
-      </c>
-      <c r="J35" t="inlineStr">
-        <is>
-          <t>23748000049202418</t>
-        </is>
-      </c>
-      <c r="K35" t="inlineStr">
-        <is>
-          <t>https://pncp.gov.br/app/editais/10784782000150/2024/17</t>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Reparo emergencial da parte elétrica dos alojamentos do IFMT Campus Confresa, com fornecimento de material.</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>23193.000138.2026-31</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>https://pncp.gov.br/app/editais/10784782000150/2026/21</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: atualizar links do Sistema S e alvaras para portais oficiais de compras
</commit_message>
<xml_diff>
--- a/oportunidades_obras_mt.xlsx
+++ b/oportunidades_obras_mt.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L48"/>
+  <dimension ref="A1:M48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -474,6 +474,11 @@
       </c>
       <c r="L1" t="inlineStr">
         <is>
+          <t>Alimentador</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
           <t>Encerramento Proposta</t>
         </is>
       </c>
@@ -524,7 +529,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>https://gazetamunicipal.cuiaba.mt.gov.br/edicoes/alvara-1842-2026</t>
+          <t>https://gazetamunicipal.cuiaba.mt.gov.br/</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -532,7 +537,12 @@
           <t>🏗️ Obra Privada (Alvará)</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr"/>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Diário Oficial (Alvarás Cuiabá/VG)</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -590,6 +600,11 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
+          <t>PNCP / Compras.gov (Governo)</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
           <t>2026-08-03 08:00</t>
         </is>
       </c>
@@ -648,7 +663,12 @@
           <t>🏛️ Governo / PNCP</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr"/>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>PNCP / Compras.gov (Governo)</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -696,7 +716,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>https://gazetamunicipal.cuiaba.mt.gov.br/edicoes/alvara-1790-2026</t>
+          <t>https://gazetamunicipal.cuiaba.mt.gov.br/</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -704,7 +724,12 @@
           <t>🏗️ Obra Privada (Alvará)</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr"/>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Diário Oficial (Alvarás Cuiabá/VG)</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -762,6 +787,11 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
+          <t>PNCP / Compras.gov (Governo)</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
           <t>2026-07-24 08:30</t>
         </is>
       </c>
@@ -812,7 +842,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>https://diariomunicipal.org/mt/amm/alvara-vg-0945-2026</t>
+          <t>https://diariomunicipal.org/mt/amm/</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -820,7 +850,12 @@
           <t>🏗️ Obra Privada (Alvará)</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr"/>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Diário Oficial (Alvarás Cuiabá/VG)</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -876,7 +911,12 @@
           <t>🏛️ Governo / PNCP</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr"/>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>PNCP / Compras.gov (Governo)</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -924,7 +964,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>https://licitacoes.portaldaindustria.com.br/fiemt/lic-042-2026</t>
+          <t>https://compras.sfiemt.ind.br/Default.aspx</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -932,7 +972,12 @@
           <t>🏢 Sistema S</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr"/>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Sistema S (Sesi/Senai/Sesc/Sebrae)</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -988,7 +1033,12 @@
           <t>🏛️ Governo / PNCP</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr"/>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>PNCP / Compras.gov (Governo)</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1036,7 +1086,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>https://licitacoes.portaldaindustria.com.br/fiemt/disp-019-2026</t>
+          <t>https://compras.sfiemt.ind.br/Default.aspx</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1044,7 +1094,12 @@
           <t>🏢 Sistema S</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr"/>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Sistema S (Sesi/Senai/Sesc/Sebrae)</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1092,7 +1147,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>https://gazetamunicipal.cuiaba.mt.gov.br/edicoes/alvara-1650-2026</t>
+          <t>https://gazetamunicipal.cuiaba.mt.gov.br/</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1100,7 +1155,12 @@
           <t>🏗️ Obra Privada (Alvará)</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr"/>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Diário Oficial (Alvarás Cuiabá/VG)</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1156,7 +1216,12 @@
           <t>🏛️ Governo / PNCP</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr"/>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>PNCP / Compras.gov (Governo)</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1216,6 +1281,11 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
+          <t>PNCP / Compras.gov (Governo)</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
           <t>2026-07-03 08:00</t>
         </is>
       </c>
@@ -1266,7 +1336,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>https://www.sescmt.com.br/licitacoes/pg-008-2026</t>
+          <t>https://transparencia-mt.sesc.com.br</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1274,7 +1344,12 @@
           <t>🏢 Sistema S</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr"/>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>Sistema S (Sesi/Senai/Sesc/Sebrae)</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1322,7 +1397,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>https://diariomunicipal.org/mt/amm/alvara-vg-0820-2026</t>
+          <t>https://diariomunicipal.org/mt/amm/</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1330,7 +1405,12 @@
           <t>🏗️ Obra Privada (Alvará)</t>
         </is>
       </c>
-      <c r="L16" t="inlineStr"/>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>Diário Oficial (Alvarás Cuiabá/VG)</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1388,6 +1468,11 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
+          <t>PNCP / Compras.gov (Governo)</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
           <t>2026-06-30 08:00</t>
         </is>
       </c>
@@ -1438,7 +1523,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>https://licitacoes.portaldaindustria.com.br/fiemt/lic-031-2026</t>
+          <t>https://compras.sfiemt.ind.br/Default.aspx</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -1446,7 +1531,12 @@
           <t>🏢 Sistema S</t>
         </is>
       </c>
-      <c r="L18" t="inlineStr"/>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>Sistema S (Sesi/Senai/Sesc/Sebrae)</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1494,7 +1584,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>https://gazetamunicipal.cuiaba.mt.gov.br/edicoes/alvara-1420-2026</t>
+          <t>https://gazetamunicipal.cuiaba.mt.gov.br/</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -1502,7 +1592,12 @@
           <t>🏗️ Obra Privada (Alvará)</t>
         </is>
       </c>
-      <c r="L19" t="inlineStr"/>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>Diário Oficial (Alvarás Cuiabá/VG)</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1558,7 +1653,12 @@
           <t>🏛️ Governo / PNCP</t>
         </is>
       </c>
-      <c r="L20" t="inlineStr"/>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>PNCP / Compras.gov (Governo)</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1616,6 +1716,11 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
+          <t>PNCP / Compras.gov (Governo)</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
           <t>2026-06-11 08:00</t>
         </is>
       </c>
@@ -1674,7 +1779,12 @@
           <t>🏛️ Governo / PNCP</t>
         </is>
       </c>
-      <c r="L22" t="inlineStr"/>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>PNCP / Compras.gov (Governo)</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1732,6 +1842,11 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
+          <t>PNCP / Compras.gov (Governo)</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
           <t>2026-06-08 12:00</t>
         </is>
       </c>
@@ -1792,6 +1907,11 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
+          <t>PNCP / Compras.gov (Governo)</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
           <t>2026-06-03 08:00</t>
         </is>
       </c>
@@ -1850,7 +1970,12 @@
           <t>🏛️ Governo / PNCP</t>
         </is>
       </c>
-      <c r="L25" t="inlineStr"/>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>PNCP / Compras.gov (Governo)</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1908,6 +2033,11 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
+          <t>PNCP / Compras.gov (Governo)</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
           <t>2026-06-02 09:00</t>
         </is>
       </c>
@@ -1958,7 +2088,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>https://sebrae.com.br/sites/PortalSebrae/licitacoes/sebrae-mt-015</t>
+          <t>https://sebrae.com.br/sites/PortalSebrae/licitacoes</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -1966,7 +2096,12 @@
           <t>🏢 Sistema S</t>
         </is>
       </c>
-      <c r="L27" t="inlineStr"/>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>Sistema S (Sesi/Senai/Sesc/Sebrae)</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2022,7 +2157,12 @@
           <t>🏛️ Governo / PNCP</t>
         </is>
       </c>
-      <c r="L28" t="inlineStr"/>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>PNCP / Compras.gov (Governo)</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2080,6 +2220,11 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
+          <t>PNCP / Compras.gov (Governo)</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
           <t>2026-05-25 09:00</t>
         </is>
       </c>
@@ -2130,7 +2275,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>https://www.sescmt.com.br/licitacoes/lic-027-2026</t>
+          <t>https://transparencia-mt.sesc.com.br</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2138,7 +2283,12 @@
           <t>🏢 Sistema S</t>
         </is>
       </c>
-      <c r="L30" t="inlineStr"/>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>Sistema S (Sesi/Senai/Sesc/Sebrae)</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2195,6 +2345,11 @@
         </is>
       </c>
       <c r="L31" t="inlineStr">
+        <is>
+          <t>PNCP / Compras.gov (Governo)</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
         <is>
           <t>2026-05-22 09:00</t>
         </is>
@@ -2258,6 +2413,11 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
+          <t>PNCP / Compras.gov (Governo)</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
           <t>2026-05-14 08:00</t>
         </is>
       </c>
@@ -2319,6 +2479,11 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
+          <t>PNCP / Compras.gov (Governo)</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
           <t>2026-05-11 08:00</t>
         </is>
       </c>
@@ -2379,6 +2544,11 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
+          <t>PNCP / Compras.gov (Governo)</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
           <t>2026-05-08 08:00</t>
         </is>
       </c>
@@ -2437,7 +2607,12 @@
           <t>🏛️ Governo / PNCP</t>
         </is>
       </c>
-      <c r="L35" t="inlineStr"/>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>PNCP / Compras.gov (Governo)</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2493,7 +2668,12 @@
           <t>🏛️ Governo / PNCP</t>
         </is>
       </c>
-      <c r="L36" t="inlineStr"/>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>PNCP / Compras.gov (Governo)</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2549,7 +2729,12 @@
           <t>🏛️ Governo / PNCP</t>
         </is>
       </c>
-      <c r="L37" t="inlineStr"/>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>PNCP / Compras.gov (Governo)</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2605,7 +2790,12 @@
           <t>🏛️ Governo / PNCP</t>
         </is>
       </c>
-      <c r="L38" t="inlineStr"/>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>PNCP / Compras.gov (Governo)</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2663,6 +2853,11 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
+          <t>PNCP / Compras.gov (Governo)</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
           <t>2026-03-30 09:00</t>
         </is>
       </c>
@@ -2723,6 +2918,11 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
+          <t>PNCP / Compras.gov (Governo)</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
           <t>2026-03-20 08:00</t>
         </is>
       </c>
@@ -2783,6 +2983,11 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
+          <t>PNCP / Compras.gov (Governo)</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
           <t>2026-03-16 08:00</t>
         </is>
       </c>
@@ -2843,6 +3048,11 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
+          <t>PNCP / Compras.gov (Governo)</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
           <t>2026-03-17 08:00</t>
         </is>
       </c>
@@ -2901,7 +3111,12 @@
           <t>🏛️ Governo / PNCP</t>
         </is>
       </c>
-      <c r="L43" t="inlineStr"/>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>PNCP / Compras.gov (Governo)</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2959,6 +3174,11 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
+          <t>PNCP / Compras.gov (Governo)</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
           <t>2026-03-04 08:00</t>
         </is>
       </c>
@@ -3019,6 +3239,11 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
+          <t>PNCP / Compras.gov (Governo)</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
           <t>2026-03-10 08:00</t>
         </is>
       </c>
@@ -3077,7 +3302,12 @@
           <t>🏛️ Governo / PNCP</t>
         </is>
       </c>
-      <c r="L46" t="inlineStr"/>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>PNCP / Compras.gov (Governo)</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -3133,7 +3363,12 @@
           <t>🏛️ Governo / PNCP</t>
         </is>
       </c>
-      <c r="L47" t="inlineStr"/>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>PNCP / Compras.gov (Governo)</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -3189,7 +3424,12 @@
           <t>🏛️ Governo / PNCP</t>
         </is>
       </c>
-      <c r="L48" t="inlineStr"/>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>PNCP / Compras.gov (Governo)</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>